<commit_message>
Round 1 done. some figures not generated. rest all OK
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,22 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pantoine/code/jpe/packages/JPE-Yang-20250178/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35869899-6FB9-B64B-8370-E5F3B9D73496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -25,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="130">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -46,13 +56,393 @@
   </si>
   <si>
     <t>In-text numbers</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">9 files in BERT_prediction_resource/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>(+ CSV twins)</t>
+    </r>
+  </si>
+  <si>
+    <t>Files in code/BERT_generation</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>Table 3</t>
+  </si>
+  <si>
+    <t>Table 4</t>
+  </si>
+  <si>
+    <t>Table 5</t>
+  </si>
+  <si>
+    <t>Table 6</t>
+  </si>
+  <si>
+    <t>Table 7</t>
+  </si>
+  <si>
+    <t>Table 8</t>
+  </si>
+  <si>
+    <t>Table A1</t>
+  </si>
+  <si>
+    <t>Table A2</t>
+  </si>
+  <si>
+    <t>Table A4</t>
+  </si>
+  <si>
+    <t>Table A5</t>
+  </si>
+  <si>
+    <t>Table A6</t>
+  </si>
+  <si>
+    <t>Table A7</t>
+  </si>
+  <si>
+    <t>Table A8</t>
+  </si>
+  <si>
+    <t>Table A9</t>
+  </si>
+  <si>
+    <t>Table A10</t>
+  </si>
+  <si>
+    <t>Table A11</t>
+  </si>
+  <si>
+    <t>Table A12</t>
+  </si>
+  <si>
+    <t>Table A13</t>
+  </si>
+  <si>
+    <t>Table A14</t>
+  </si>
+  <si>
+    <t>Table A15</t>
+  </si>
+  <si>
+    <t>Table A16</t>
+  </si>
+  <si>
+    <t>Table A17</t>
+  </si>
+  <si>
+    <t>Table A18</t>
+  </si>
+  <si>
+    <t>Table A19</t>
+  </si>
+  <si>
+    <t>Table A20</t>
+  </si>
+  <si>
+    <t>Table A21</t>
+  </si>
+  <si>
+    <t>Table A22</t>
+  </si>
+  <si>
+    <t>Table A23</t>
+  </si>
+  <si>
+    <t>Table A24</t>
+  </si>
+  <si>
+    <t>Table A25</t>
+  </si>
+  <si>
+    <t>Table A26</t>
+  </si>
+  <si>
+    <t>Table A27</t>
+  </si>
+  <si>
+    <t>Table A28</t>
+  </si>
+  <si>
+    <t>Table A29</t>
+  </si>
+  <si>
+    <t>Table A30</t>
+  </si>
+  <si>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>Figure 4</t>
+  </si>
+  <si>
+    <t>Figure A1</t>
+  </si>
+  <si>
+    <t>Figure A2</t>
+  </si>
+  <si>
+    <t>Figure A3</t>
+  </si>
+  <si>
+    <t>Figure A4</t>
+  </si>
+  <si>
+    <t>Figure A5</t>
+  </si>
+  <si>
+    <t>Figure A6</t>
+  </si>
+  <si>
+    <t>Figure A7</t>
+  </si>
+  <si>
+    <t>Figure A8</t>
+  </si>
+  <si>
+    <t>Figure A9</t>
+  </si>
+  <si>
+    <t>Figure A10</t>
+  </si>
+  <si>
+    <t>Figure A11</t>
+  </si>
+  <si>
+    <t>Figure A12</t>
+  </si>
+  <si>
+    <t>Figure A13</t>
+  </si>
+  <si>
+    <t>Figure A14</t>
+  </si>
+  <si>
+    <t>Figure A15</t>
+  </si>
+  <si>
+    <t>Figure A16</t>
+  </si>
+  <si>
+    <t>Figure A17</t>
+  </si>
+  <si>
+    <t>code/tables/table_1.py</t>
+  </si>
+  <si>
+    <t>code/tables/table_A1.py</t>
+  </si>
+  <si>
+    <t>code/tables/table_2.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_3.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_4.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_5.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_6.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_7.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_8.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A2.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A4.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A5.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A6.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A7.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A8.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A9.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A10.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A11.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A12.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A13.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A14.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A15.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A16.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A17.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A18.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A20.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A30.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A21.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A22.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A23.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A24.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A25.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A26.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A27.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A28.do</t>
+  </si>
+  <si>
+    <t>code/tables/table_A29.do</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>code/figures/figure_1.py</t>
+  </si>
+  <si>
+    <t>code/figures/figure_2.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_3.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_4.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A1.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A2.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A3.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A4.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A5.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A6.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A7.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A8.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A9.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A10.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A11.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A12.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A13.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A14.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A15.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A16.do</t>
+  </si>
+  <si>
+    <t>code/figures/figure_A17.do</t>
+  </si>
+  <si>
+    <t>Tabe A3</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>No script (textual data)</t>
+  </si>
+  <si>
+    <t>No (skipped)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -64,6 +454,24 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Monaco"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -89,7 +497,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -100,6 +508,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,11 +843,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -460,51 +869,871 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
+    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>126</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C14" t="s">
+        <v>104</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" t="s">
+        <v>104</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" t="s">
+        <v>104</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" t="s">
+        <v>104</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C25" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>31</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" t="s">
+        <v>104</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" t="s">
+        <v>104</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" t="s">
+        <v>104</v>
+      </c>
+      <c r="D30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" t="s">
+        <v>104</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" t="s">
+        <v>104</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C34" t="s">
+        <v>104</v>
+      </c>
+      <c r="D34" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" t="s">
+        <v>104</v>
+      </c>
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" t="s">
+        <v>104</v>
+      </c>
+      <c r="D37" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" t="s">
+        <v>104</v>
+      </c>
+      <c r="D38" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" t="s">
+        <v>104</v>
+      </c>
+      <c r="D40" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C41" t="s">
+        <v>104</v>
+      </c>
+      <c r="D41" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>47</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C42" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>48</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" t="s">
+        <v>104</v>
+      </c>
+      <c r="D43" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>49</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C44" t="s">
+        <v>104</v>
+      </c>
+      <c r="D44" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>50</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" t="s">
+        <v>104</v>
+      </c>
+      <c r="D45" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>51</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C46" t="s">
+        <v>104</v>
+      </c>
+      <c r="D46" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>52</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C47" t="s">
+        <v>104</v>
+      </c>
+      <c r="D47" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>53</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C48" t="s">
+        <v>104</v>
+      </c>
+      <c r="D48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>54</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C49" t="s">
+        <v>104</v>
+      </c>
+      <c r="D49" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>55</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C50" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C51" t="s">
+        <v>104</v>
+      </c>
+      <c r="D51" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>57</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C52" t="s">
+        <v>104</v>
+      </c>
+      <c r="D52" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>58</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C53" t="s">
+        <v>104</v>
+      </c>
+      <c r="D53" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C54" t="s">
+        <v>104</v>
+      </c>
+      <c r="D54" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>60</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C55" t="s">
+        <v>104</v>
+      </c>
+      <c r="D55" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C56" t="s">
+        <v>104</v>
+      </c>
+      <c r="D56" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C57" t="s">
+        <v>104</v>
+      </c>
+      <c r="D57" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>63</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C58" t="s">
+        <v>104</v>
+      </c>
+      <c r="D58" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C59" t="s">
+        <v>104</v>
+      </c>
+      <c r="D59" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>65</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C60" t="s">
+        <v>104</v>
+      </c>
+      <c r="D60" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C61" t="s">
+        <v>104</v>
+      </c>
+      <c r="D61" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>67</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C62" t="s">
+        <v>104</v>
+      </c>
+      <c r="D62" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C63" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
-      </c>
+      <c r="D63" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>